<commit_message>
Daily slate 2026-06-17 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-15.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-15.xlsx
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="E4" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F4" t="n">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="G4" t="n">
-        <v>39.3</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="5">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E7" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F7" t="n">
         <v>31</v>
       </c>
       <c r="G7" t="n">
-        <v>53</v>
+        <v>54.4</v>
       </c>
     </row>
     <row r="8">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E9" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F9" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G9" t="n">
-        <v>54.7</v>
+        <v>56.1</v>
       </c>
     </row>
     <row r="10">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>840</v>
+        <v>890</v>
       </c>
       <c r="E11" t="n">
-        <v>474</v>
+        <v>487</v>
       </c>
       <c r="F11" t="n">
-        <v>366</v>
+        <v>403</v>
       </c>
       <c r="G11" t="n">
-        <v>56.4</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E12" t="n">
         <v>100</v>
       </c>
       <c r="F12" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G12" t="n">
-        <v>62.1</v>
+        <v>61.7</v>
       </c>
     </row>
     <row r="13">
@@ -816,16 +816,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="E14" t="n">
         <v>58</v>
       </c>
       <c r="F14" t="n">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="G14" t="n">
-        <v>22.7</v>
+        <v>22.1</v>
       </c>
     </row>
     <row r="15">
@@ -845,16 +845,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="E15" t="n">
         <v>66</v>
       </c>
       <c r="F15" t="n">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="G15" t="n">
-        <v>17.4</v>
+        <v>17.1</v>
       </c>
     </row>
     <row r="16">
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3087</v>
+        <v>3294</v>
       </c>
       <c r="E17" t="n">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="F17" t="n">
-        <v>2491</v>
+        <v>2683</v>
       </c>
       <c r="G17" t="n">
-        <v>19.3</v>
+        <v>18.5</v>
       </c>
     </row>
   </sheetData>
@@ -1531,16 +1531,16 @@
         <v>181</v>
       </c>
       <c r="D7" t="n">
-        <v>56.4</v>
+        <v>54.7</v>
       </c>
       <c r="E7" t="n">
-        <v>840</v>
+        <v>890</v>
       </c>
       <c r="F7" t="n">
-        <v>62.1</v>
+        <v>61.7</v>
       </c>
       <c r="G7" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H7" t="n">
         <v>43</v>
@@ -1549,16 +1549,16 @@
         <v>151</v>
       </c>
       <c r="J7" t="n">
-        <v>22.7</v>
+        <v>22.1</v>
       </c>
       <c r="K7" t="n">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="L7" t="n">
-        <v>17.4</v>
+        <v>17.1</v>
       </c>
       <c r="M7" t="n">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="N7" t="n">
         <v>15.4</v>
@@ -1567,10 +1567,10 @@
         <v>272</v>
       </c>
       <c r="P7" t="n">
-        <v>19.3</v>
+        <v>18.5</v>
       </c>
       <c r="Q7" t="n">
-        <v>3087</v>
+        <v>3294</v>
       </c>
       <c r="R7" t="n">
         <v>33.5</v>
@@ -1579,10 +1579,10 @@
         <v>334</v>
       </c>
       <c r="T7" t="n">
-        <v>39.3</v>
+        <v>38.6</v>
       </c>
       <c r="U7" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="W7" t="n">
         <v>0</v>
@@ -1606,16 +1606,16 @@
         <v>41</v>
       </c>
       <c r="AD7" t="n">
-        <v>53</v>
+        <v>54.4</v>
       </c>
       <c r="AE7" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="AF7" t="n">
-        <v>54.7</v>
+        <v>56.1</v>
       </c>
       <c r="AG7" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily slate 2026-06-18 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-06-15.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-06-15.xlsx
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E7" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F7" t="n">
         <v>31</v>
       </c>
       <c r="G7" t="n">
-        <v>54.4</v>
+        <v>55.1</v>
       </c>
     </row>
     <row r="8">
@@ -671,16 +671,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E9" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F9" t="n">
         <v>25</v>
       </c>
       <c r="G9" t="n">
-        <v>56.1</v>
+        <v>56.9</v>
       </c>
     </row>
     <row r="10">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>890</v>
+        <v>893</v>
       </c>
       <c r="E11" t="n">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="F11" t="n">
         <v>403</v>
       </c>
       <c r="G11" t="n">
-        <v>54.7</v>
+        <v>54.9</v>
       </c>
     </row>
     <row r="12">
@@ -758,16 +758,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E12" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F12" t="n">
         <v>62</v>
       </c>
       <c r="G12" t="n">
-        <v>61.7</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13">
@@ -845,13 +845,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E15" t="n">
         <v>66</v>
       </c>
       <c r="F15" t="n">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G15" t="n">
         <v>17.1</v>
@@ -903,16 +903,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3294</v>
+        <v>3301</v>
       </c>
       <c r="E17" t="n">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F17" t="n">
-        <v>2683</v>
+        <v>2688</v>
       </c>
       <c r="G17" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
     </row>
   </sheetData>
@@ -1531,16 +1531,16 @@
         <v>181</v>
       </c>
       <c r="D7" t="n">
-        <v>54.7</v>
+        <v>54.9</v>
       </c>
       <c r="E7" t="n">
-        <v>890</v>
+        <v>893</v>
       </c>
       <c r="F7" t="n">
-        <v>61.7</v>
+        <v>62</v>
       </c>
       <c r="G7" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H7" t="n">
         <v>43</v>
@@ -1558,7 +1558,7 @@
         <v>17.1</v>
       </c>
       <c r="M7" t="n">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="N7" t="n">
         <v>15.4</v>
@@ -1567,10 +1567,10 @@
         <v>272</v>
       </c>
       <c r="P7" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>3294</v>
+        <v>3301</v>
       </c>
       <c r="R7" t="n">
         <v>33.5</v>
@@ -1606,16 +1606,16 @@
         <v>41</v>
       </c>
       <c r="AD7" t="n">
-        <v>54.4</v>
+        <v>55.1</v>
       </c>
       <c r="AE7" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AF7" t="n">
-        <v>56.1</v>
+        <v>56.9</v>
       </c>
       <c r="AG7" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>